<commit_message>
Fix NetworkMonitorService device selection: prioritize Windows loopback, then Docker custom bridge (br-xxxxx), then docker0
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/cuongnhhe186494/TC1/GradeDetail.xlsx
+++ b/Submit/Results/cuongnhhe186494/TC1/GradeDetail.xlsx
@@ -162,13 +162,13 @@
     <x:t>NetworkResult</x:t>
   </x:si>
   <x:si>
-    <x:t>2025-12-02 15:22:36</x:t>
+    <x:t>2025-12-02 15:32:46</x:t>
   </x:si>
   <x:si>
     <x:t>TCP</x:t>
   </x:si>
   <x:si>
-    <x:t>127.0.0.1:50694</x:t>
+    <x:t>127.0.0.1:46148</x:t>
   </x:si>
   <x:si>
     <x:t>127.0.0.1:8000</x:t>

</xml_diff>

<commit_message>
Sync CLI and UI: match testkit Network sheet format, add FileMaster zip extraction
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/cuongnhhe186494/TC1/GradeDetail.xlsx
+++ b/Submit/Results/cuongnhhe186494/TC1/GradeDetail.xlsx
@@ -144,31 +144,13 @@
     <x:t>DestinationRole</x:t>
   </x:si>
   <x:si>
-    <x:t>ActualFlags</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ActualState</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ActualSourceRole</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ActualDestRole</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ActualData</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NetworkResult</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2025-12-02 15:32:46</x:t>
+    <x:t>2025-12-02 15:59:26</x:t>
   </x:si>
   <x:si>
     <x:t>TCP</x:t>
   </x:si>
   <x:si>
-    <x:t>127.0.0.1:46148</x:t>
+    <x:t>127.0.0.1:39976</x:t>
   </x:si>
   <x:si>
     <x:t>127.0.0.1:8000</x:t>
@@ -972,7 +954,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:P8"/>
+  <x:dimension ref="A1:J8"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="5.710625" style="0" customWidth="1"/>
@@ -984,15 +966,9 @@
     <x:col min="8" max="8" width="4.996339" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="10.853482" style="0" customWidth="1"/>
     <x:col min="10" max="10" width="15.139196" style="0" customWidth="1"/>
-    <x:col min="11" max="11" width="10.853482" style="0" customWidth="1"/>
-    <x:col min="12" max="12" width="29.996339" style="0" customWidth="1"/>
-    <x:col min="13" max="13" width="16.424911" style="0" customWidth="1"/>
-    <x:col min="14" max="14" width="14.424911" style="0" customWidth="1"/>
-    <x:col min="15" max="15" width="10.567768" style="0" customWidth="1"/>
-    <x:col min="16" max="16" width="14.139196" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:16" s="1" customFormat="1">
+    <x:row r="1" spans="1:10" s="1" customFormat="1">
       <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -1023,373 +999,229 @@
       <x:c r="J1" s="1" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="K1" s="1" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="L1" s="1" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="M1" s="1" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="N1" s="1" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="O1" s="1" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="P1" s="1" t="s">
-        <x:v>46</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:16">
+    </x:row>
+    <x:row r="2" spans="1:10">
       <x:c r="A2" s="0">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="H2" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I2" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J2" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="K2" s="0" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="L2" s="0" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="M2" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="N2" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="O2" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="P2" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:16">
+        <x:v>48</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:10">
       <x:c r="A3" s="0">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
         <x:v>50</x:v>
-      </x:c>
-      <x:c r="E3" s="0" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="F3" s="0" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="G3" s="0" t="s">
-        <x:v>56</x:v>
       </x:c>
       <x:c r="H3" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I3" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="J3" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="K3" s="0" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="L3" s="0" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="M3" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="N3" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="O3" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="P3" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:16">
+        <x:v>47</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:10">
       <x:c r="A4" s="0">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="H4" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I4" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J4" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="K4" s="0" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="L4" s="0" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="M4" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="N4" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="O4" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="P4" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:16">
+        <x:v>48</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:10">
       <x:c r="A5" s="0">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="G5" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="H5" s="2" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="I5" s="0" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="C5" s="0" t="s">
+      <x:c r="J5" s="0" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="D5" s="0" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="E5" s="0" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="F5" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="G5" s="0" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="H5" s="2" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I5" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="J5" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="K5" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="L5" s="0" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="M5" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="N5" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="O5" s="2" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="P5" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:16">
+    </x:row>
+    <x:row r="6" spans="1:10">
       <x:c r="A6" s="0">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="G6" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="H6" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I6" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="J6" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="K6" s="0" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="L6" s="0" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="M6" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="N6" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="O6" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="P6" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:16">
+        <x:v>47</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:10">
       <x:c r="A7" s="0">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="G7" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="H7" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="I7" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="J7" s="0" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="C7" s="0" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="D7" s="0" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="E7" s="0" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="F7" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="G7" s="0" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="H7" s="0" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="I7" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="J7" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="K7" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="L7" s="0" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="M7" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="N7" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="O7" s="0" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="P7" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:16">
+    </x:row>
+    <x:row r="8" spans="1:10">
       <x:c r="A8" s="0">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="F8" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="G8" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="H8" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I8" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J8" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="K8" s="0" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="L8" s="0" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="M8" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="N8" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="O8" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="P8" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>